<commit_message>
modulo de inventario y cobros
</commit_message>
<xml_diff>
--- a/data/pedidos_2026-08-08.xlsx
+++ b/data/pedidos_2026-08-08.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedidos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Pedidos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,49 +454,359 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Grabado (Si/No)</t>
+          <t>Precio total</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Mensaje del grabado</t>
+          <t>Pagado (Si/No)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Precio total</t>
+          <t>Fecha de entrega</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>Pagado (Si/No)</t>
+          <t>Observaciones</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Fecha de entrega</t>
+          <t>Numero de emergencia</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
-          <t>Observaciones</t>
+          <t>Estado subida</t>
         </is>
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>Numero de emergencia</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>Estado subida</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
           <t>Error</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1. Karla Saraí Martinez Arteaga</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>74056500</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>San Salvador</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>AGUILARES</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Gasolinera Texaco Aguilares</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Gasolinera Texaco Aguilares</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Casio retro black + bolsa de regalo</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>PAGADO</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2. Edwin Milton Hernández Hernández</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>75881415</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>La Paz</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SAN PEDRO MASAHUAT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Calle hacia playa Las Hojas, El Achiotal</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Frente a la bomba de agua</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Promocion lente aviador negro y Wood negro</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar la entrega</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3. Eliza Osorio</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>70188670</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>La Libertad</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SAN JUAN OPICO</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Pje. Jazmin, Sitio del Niño</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Centro Urbano de Bienestar y Oportunidades (CUBO) Ing. Rigoberto Orellana</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>wood cafe; wood negro</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ENTREGAR DESPUES DE LAS 12PM</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4. Gerardo Munguia</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>77520030</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>San Miguel</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SAN MIGUEL</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Agencia de express san miguel</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Envio de agencia a agencia</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Casio world plata</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Envio de agencia a agencia</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>5. Francisco Javier Avilés Martínez</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>76516434</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>La Libertad</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>QUEZALTEPEQUE</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>parqué central</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>parqué central</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>casio world</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Contactar al cliente para coordinar la entrega</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>